<commit_message>
gcomp/psdash: extend QA coverage, refine detection and bootstrap logic
</commit_message>
<xml_diff>
--- a/psdash/demo/psdash_report.xlsx
+++ b/psdash/demo/psdash_report.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="200" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="200" uniqueCount="141">
   <si>
     <t>PS Overlap</t>
   </si>
@@ -427,7 +427,13 @@
     <t>manual</t>
   </si>
   <si>
-    <t>PASS</t>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>weights</t>
   </si>
   <si>
     <t>10</t>
@@ -1225,7 +1231,7 @@
         <v>129</v>
       </c>
       <c r="B8" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9">
@@ -1233,7 +1239,7 @@
         <v>130</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10">
@@ -1241,7 +1247,7 @@
         <v>131</v>
       </c>
       <c r="B10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11">
@@ -1249,7 +1255,7 @@
         <v>132</v>
       </c>
       <c r="B11" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
fix(psdash,kmplot,pkgtransfer): sync release fixes and add pkgtransfe...
Bump kmplot to 1.2.6: _kmplot_risktable.ado adds TOPTimeaxis to
xaxis(1 2) the number-at-risk table above a horizontal separator and
raise its label size from vsmall to small, matching kmplot.ado,
kmplot.sthlp, and README.md. Bump psdash to 1.6.7 across its .ado
helpers with README synced. Add pkgtransfer/README.md and new
demo/console_*.md walkthroughs plus demo/demo_pkgtransfer.do. Add
kmplot/qa/test_kmplot_v126.do regression coverage and update
qa/README.md and qa/run_all.do to include it. Regenerate demo
artifacts across codescan, finegray, iivw, and kmplot
(codescan_results.xlsx, prevalence_chart.png, finegray_cif.png,
iivw_psdash_dashboard.png, iivw_psdash_final_weights.png,
iivw_reporting_exports.xlsx, iivw_results.xlsx, and the km_*.png set)
to reflect current output. Update the root README.md version/date
badges for psdash and kmplot.
</commit_message>
<xml_diff>
--- a/psdash/demo/psdash_report.xlsx
+++ b/psdash/demo/psdash_report.xlsx
@@ -2727,7 +2727,7 @@
         <v>0.0133601195235551</v>
       </c>
       <c r="J3" s="53">
-        <v>1.0070175475116769</v>
+        <v>1.006001716637021</v>
       </c>
       <c r="K3" s="54">
         <v>0.050854877187559502</v>
@@ -2744,10 +2744,10 @@
         <v>0.37751004016064249</v>
       </c>
       <c r="D4" s="57">
-        <v>0.43031695072119203</v>
+        <v>0.43094226089634691</v>
       </c>
       <c r="E4" s="58">
-        <v>1.028603636082803</v>
+        <v>1.030876909735525</v>
       </c>
       <c r="F4" s="59">
         <v>0.2105117384237494</v>
@@ -2759,10 +2759,10 @@
         <v>0.52192770278459788</v>
       </c>
       <c r="I4" s="62">
-        <v>0.0011499000107072</v>
+        <v>0.0011515709748091</v>
       </c>
       <c r="J4" s="63">
-        <v>0.99769489764372021</v>
+        <v>0.99989986119304719</v>
       </c>
       <c r="K4" s="64">
         <v>0.00056253291872829995</v>
@@ -2797,7 +2797,7 @@
         <v>0.013785947066266801</v>
       </c>
       <c r="J5" s="73">
-        <v>1.0726598498761111</v>
+        <v>1.0715778022035549</v>
       </c>
       <c r="K5" s="74">
         <v>0.0447537937716748</v>
@@ -2832,7 +2832,7 @@
         <v>0.0182255436196882</v>
       </c>
       <c r="J6" s="83">
-        <v>1.0508027094953121</v>
+        <v>1.049742710254866</v>
       </c>
       <c r="K6" s="84">
         <v>0.093744814098041002</v>
@@ -2867,7 +2867,7 @@
         <v>0.047032989657052</v>
       </c>
       <c r="J7" s="93">
-        <v>0.99087308437154431</v>
+        <v>0.98987353925491961</v>
       </c>
       <c r="K7" s="94">
         <v>0.0376989109603907</v>

</xml_diff>